<commit_message>
feat: maj 24 ravitaillements, barriere finale 83h et barrieres horaires imposees
</commit_message>
<xml_diff>
--- a/OrgaTrail_Modele_Ravitaillements.xlsx
+++ b/OrgaTrail_Modele_Ravitaillements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chris\Desktop\Mes applis\apporgatrail\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB550572-5AB4-437E-9F96-C671EC56C09A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6867182C-6BF3-4B1F-AD0E-D86F6B30CFEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="59">
   <si>
     <t>N°</t>
   </si>
@@ -84,166 +84,124 @@
     <t>Camphrier</t>
   </si>
   <si>
-    <t>10.447</t>
-  </si>
-  <si>
     <t>COMPLET</t>
   </si>
   <si>
     <t>Foc foc</t>
   </si>
   <si>
-    <t>25.021</t>
+    <t>ZONE_BLANCHE</t>
   </si>
   <si>
     <t>Parking nez de boeuf</t>
   </si>
   <si>
-    <t>40.526</t>
-  </si>
-  <si>
-    <t>Champ de foire</t>
-  </si>
-  <si>
-    <t>47.749</t>
-  </si>
-  <si>
     <t>Horloge</t>
   </si>
   <si>
-    <t>54.474</t>
+    <t>Gd bassin</t>
+  </si>
+  <si>
+    <t>HELICO</t>
+  </si>
+  <si>
+    <t>Mare a boue</t>
   </si>
   <si>
     <t>PIETON</t>
   </si>
   <si>
-    <t>Gd bassin</t>
-  </si>
-  <si>
-    <t>58.672</t>
-  </si>
-  <si>
-    <t>Mare a boue</t>
-  </si>
-  <si>
-    <t>66.135</t>
-  </si>
-  <si>
-    <t>ZONE_BLANCHE</t>
-  </si>
-  <si>
     <t>Parking marsoin</t>
   </si>
   <si>
-    <t>74.686</t>
-  </si>
-  <si>
-    <t>HELICO</t>
+    <t>INTERDIT</t>
   </si>
   <si>
     <t>Hell bourg</t>
   </si>
   <si>
-    <t>87.522</t>
+    <t>BASE_VIE</t>
   </si>
   <si>
     <t>Gite dufour 1</t>
   </si>
   <si>
-    <t>95.166</t>
-  </si>
-  <si>
     <t>EAU</t>
   </si>
   <si>
     <t>Sommet piton</t>
   </si>
   <si>
-    <t>98.214</t>
-  </si>
-  <si>
     <t>Gite dufour 2</t>
   </si>
   <si>
-    <t>101.27</t>
-  </si>
-  <si>
     <t>Cilaos</t>
   </si>
   <si>
-    <t>110.811</t>
-  </si>
-  <si>
-    <t>BASE_VIE</t>
-  </si>
-  <si>
     <t>Pied taibit</t>
   </si>
   <si>
-    <t>117.97</t>
-  </si>
-  <si>
     <t>Marla</t>
   </si>
   <si>
-    <t>124.134</t>
-  </si>
-  <si>
     <t>La nouvelle</t>
   </si>
   <si>
-    <t>130.827</t>
-  </si>
-  <si>
     <t>Roche plate</t>
   </si>
   <si>
-    <t>140.049</t>
-  </si>
-  <si>
     <t>Maido</t>
   </si>
   <si>
-    <t>147.476</t>
-  </si>
-  <si>
     <t>Tamarin</t>
   </si>
   <si>
-    <t>162.201</t>
-  </si>
-  <si>
     <t>Piton oranger</t>
   </si>
   <si>
-    <t>172.308</t>
-  </si>
-  <si>
     <t>Halte la</t>
   </si>
   <si>
-    <t>189.71</t>
-  </si>
-  <si>
     <t>Cap noir</t>
   </si>
   <si>
-    <t>197.898</t>
-  </si>
-  <si>
     <t>Colorado</t>
   </si>
   <si>
-    <t>213.424</t>
-  </si>
-  <si>
     <t>La Redoute - Saint-Denis (ARRIVÉE)</t>
   </si>
   <si>
-    <t>220.341</t>
-  </si>
-  <si>
-    <t>INTERDIT</t>
+    <t>jeu 09:00</t>
+  </si>
+  <si>
+    <t>jeu 16:00</t>
+  </si>
+  <si>
+    <t>dim 14:30</t>
+  </si>
+  <si>
+    <t>ven 00:15</t>
+  </si>
+  <si>
+    <t>ven 05:15</t>
+  </si>
+  <si>
+    <t>ven 09:15</t>
+  </si>
+  <si>
+    <t>ven 23:00</t>
+  </si>
+  <si>
+    <t>sam 01:30</t>
+  </si>
+  <si>
+    <t>sam 13:45</t>
+  </si>
+  <si>
+    <t>dim 09:00</t>
+  </si>
+  <si>
+    <t>ven 02:00</t>
   </si>
 </sst>
 </file>
@@ -620,11 +578,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.875" customWidth="1"/>
-    <col min="2" max="2" width="32.875" customWidth="1"/>
+    <col min="2" max="2" width="34.875" customWidth="1"/>
     <col min="3" max="3" width="15.875" customWidth="1"/>
     <col min="4" max="4" width="18.875" customWidth="1"/>
     <col min="5" max="5" width="15.875" customWidth="1"/>
@@ -635,7 +593,7 @@
     <col min="10" max="11" width="10.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -670,7 +628,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -680,9 +638,6 @@
       <c r="C2">
         <v>0</v>
       </c>
-      <c r="D2" t="s">
-        <v>12</v>
-      </c>
       <c r="E2" t="s">
         <v>13</v>
       </c>
@@ -705,21 +660,21 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
         <v>18</v>
       </c>
-      <c r="C3" t="s">
-        <v>19</v>
+      <c r="C3">
+        <v>10.446999999999999</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="E3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F3">
         <v>2</v>
@@ -740,21 +695,21 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" t="s">
-        <v>22</v>
+        <v>20</v>
+      </c>
+      <c r="C4">
+        <v>25.021000000000001</v>
       </c>
       <c r="D4" t="s">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="E4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F4">
         <v>4</v>
@@ -766,7 +721,7 @@
         <v>14</v>
       </c>
       <c r="I4" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="J4" t="s">
         <v>16</v>
@@ -775,21 +730,18 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" t="s">
-        <v>24</v>
-      </c>
-      <c r="D5" t="s">
-        <v>12</v>
+        <v>22</v>
+      </c>
+      <c r="C5">
+        <v>40.526000000000003</v>
       </c>
       <c r="E5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F5">
         <v>3</v>
@@ -810,24 +762,24 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C6" t="s">
-        <v>26</v>
+        <v>23</v>
+      </c>
+      <c r="C6">
+        <v>54.473999999999997</v>
       </c>
       <c r="D6" t="s">
-        <v>12</v>
+        <v>51</v>
       </c>
       <c r="E6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G6">
         <v>15</v>
@@ -839,176 +791,176 @@
         <v>15</v>
       </c>
       <c r="J6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7" t="s">
-        <v>28</v>
+        <v>24</v>
+      </c>
+      <c r="C7">
+        <v>58.671999999999997</v>
       </c>
       <c r="D7" t="s">
-        <v>12</v>
+        <v>58</v>
       </c>
       <c r="E7" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="F7">
         <v>2</v>
       </c>
       <c r="G7">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="H7" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="I7" t="s">
         <v>15</v>
       </c>
       <c r="J7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K7" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" t="s">
-        <v>31</v>
+        <v>26</v>
+      </c>
+      <c r="C8">
+        <v>66.135000000000005</v>
       </c>
       <c r="D8" t="s">
-        <v>12</v>
+        <v>52</v>
       </c>
       <c r="E8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F8">
         <v>2</v>
       </c>
       <c r="G8">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="H8" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="I8" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="J8" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" t="s">
-        <v>33</v>
+        <v>28</v>
+      </c>
+      <c r="C9">
+        <v>74.686000000000007</v>
       </c>
       <c r="D9" t="s">
         <v>12</v>
       </c>
       <c r="E9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F9">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G9">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H9" t="s">
         <v>29</v>
       </c>
       <c r="I9" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="J9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>35</v>
-      </c>
-      <c r="C10" t="s">
-        <v>36</v>
+        <v>30</v>
+      </c>
+      <c r="C10">
+        <v>87.522000000000006</v>
       </c>
       <c r="D10" t="s">
-        <v>12</v>
+        <v>53</v>
       </c>
       <c r="E10" t="s">
+        <v>31</v>
+      </c>
+      <c r="F10">
+        <v>3</v>
+      </c>
+      <c r="G10">
         <v>20</v>
       </c>
-      <c r="F10">
-        <v>5</v>
-      </c>
-      <c r="G10">
-        <v>30</v>
-      </c>
       <c r="H10" t="s">
-        <v>72</v>
+        <v>14</v>
       </c>
       <c r="I10" t="s">
         <v>15</v>
       </c>
       <c r="J10" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K10" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>38</v>
-      </c>
-      <c r="C11" t="s">
-        <v>39</v>
+        <v>32</v>
+      </c>
+      <c r="C11">
+        <v>95.165999999999997</v>
       </c>
       <c r="D11" t="s">
         <v>12</v>
       </c>
       <c r="E11" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="F11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G11">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="H11" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="I11" t="s">
         <v>15</v>
@@ -1020,65 +972,65 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" t="s">
-        <v>41</v>
+        <v>34</v>
+      </c>
+      <c r="C12">
+        <v>98.213999999999999</v>
       </c>
       <c r="D12" t="s">
         <v>12</v>
       </c>
       <c r="E12" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="F12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G12">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="H12" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="I12" t="s">
         <v>15</v>
       </c>
       <c r="J12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K12" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>43</v>
-      </c>
-      <c r="C13" t="s">
-        <v>44</v>
+        <v>35</v>
+      </c>
+      <c r="C13">
+        <v>101.27</v>
       </c>
       <c r="D13" t="s">
         <v>12</v>
       </c>
       <c r="E13" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="F13">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G13">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H13" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="I13" t="s">
         <v>15</v>
@@ -1090,30 +1042,30 @@
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14">
+        <v>110.81100000000001</v>
+      </c>
+      <c r="D14" t="s">
+        <v>54</v>
+      </c>
+      <c r="E14" t="s">
+        <v>31</v>
+      </c>
+      <c r="F14">
+        <v>12</v>
+      </c>
+      <c r="G14">
         <v>45</v>
       </c>
-      <c r="C14" t="s">
-        <v>46</v>
-      </c>
-      <c r="D14" t="s">
-        <v>12</v>
-      </c>
-      <c r="E14" t="s">
-        <v>42</v>
-      </c>
-      <c r="F14">
-        <v>2</v>
-      </c>
-      <c r="G14">
-        <v>10</v>
-      </c>
       <c r="H14" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="I14" t="s">
         <v>15</v>
@@ -1122,30 +1074,30 @@
         <v>16</v>
       </c>
       <c r="K14" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>47</v>
-      </c>
-      <c r="C15" t="s">
-        <v>48</v>
+        <v>37</v>
+      </c>
+      <c r="C15">
+        <v>117.97</v>
       </c>
       <c r="D15" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="E15" t="s">
-        <v>49</v>
+        <v>19</v>
       </c>
       <c r="F15">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="G15">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="H15" t="s">
         <v>14</v>
@@ -1154,72 +1106,69 @@
         <v>15</v>
       </c>
       <c r="J15" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K15" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>50</v>
-      </c>
-      <c r="C16" t="s">
-        <v>51</v>
-      </c>
-      <c r="D16" t="s">
-        <v>12</v>
+        <v>38</v>
+      </c>
+      <c r="C16">
+        <v>124.134</v>
       </c>
       <c r="E16" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F16">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G16">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="H16" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="I16" t="s">
         <v>15</v>
       </c>
       <c r="J16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K16" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>52</v>
-      </c>
-      <c r="C17" t="s">
-        <v>53</v>
+        <v>39</v>
+      </c>
+      <c r="C17">
+        <v>130.827</v>
       </c>
       <c r="D17" t="s">
         <v>12</v>
       </c>
       <c r="E17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F17">
         <v>4</v>
       </c>
       <c r="G17">
+        <v>20</v>
+      </c>
+      <c r="H17" t="s">
         <v>25</v>
       </c>
-      <c r="H17" t="s">
-        <v>37</v>
-      </c>
       <c r="I17" t="s">
         <v>15</v>
       </c>
@@ -1230,135 +1179,135 @@
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>54</v>
-      </c>
-      <c r="C18" t="s">
-        <v>55</v>
+        <v>40</v>
+      </c>
+      <c r="C18">
+        <v>140.04900000000001</v>
       </c>
       <c r="D18" t="s">
         <v>12</v>
       </c>
       <c r="E18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F18">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G18">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H18" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="I18" t="s">
         <v>15</v>
       </c>
       <c r="J18" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K18" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19" t="s">
+        <v>41</v>
+      </c>
+      <c r="C19">
+        <v>147.476</v>
+      </c>
+      <c r="D19" t="s">
         <v>56</v>
       </c>
-      <c r="C19" t="s">
-        <v>57</v>
-      </c>
-      <c r="D19" t="s">
-        <v>12</v>
-      </c>
       <c r="E19" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F19">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G19">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="H19" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="I19" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="J19" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K19" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>58</v>
-      </c>
-      <c r="C20" t="s">
-        <v>59</v>
+        <v>42</v>
+      </c>
+      <c r="C20">
+        <v>162.20099999999999</v>
       </c>
       <c r="D20" t="s">
         <v>12</v>
       </c>
       <c r="E20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F20">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G20">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="H20" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="I20" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="J20" t="s">
         <v>16</v>
       </c>
       <c r="K20" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>60</v>
-      </c>
-      <c r="C21" t="s">
-        <v>61</v>
+        <v>43</v>
+      </c>
+      <c r="C21">
+        <v>172.30799999999999</v>
       </c>
       <c r="D21" t="s">
         <v>12</v>
       </c>
       <c r="E21" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F21">
         <v>2</v>
       </c>
       <c r="G21">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="H21" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="I21" t="s">
         <v>15</v>
@@ -1370,97 +1319,94 @@
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>62</v>
-      </c>
-      <c r="C22" t="s">
-        <v>63</v>
+        <v>44</v>
+      </c>
+      <c r="C22">
+        <v>189.71</v>
       </c>
       <c r="D22" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="E22" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="F22">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G22">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="H22" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="I22" t="s">
         <v>15</v>
       </c>
       <c r="J22" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K22" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>64</v>
-      </c>
-      <c r="C23" t="s">
-        <v>65</v>
-      </c>
-      <c r="D23" t="s">
-        <v>12</v>
+        <v>45</v>
+      </c>
+      <c r="C23">
+        <v>197.898</v>
       </c>
       <c r="E23" t="s">
-        <v>49</v>
+        <v>19</v>
       </c>
       <c r="F23">
+        <v>3</v>
+      </c>
+      <c r="G23">
         <v>10</v>
       </c>
-      <c r="G23">
-        <v>55</v>
-      </c>
       <c r="H23" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="I23" t="s">
         <v>15</v>
       </c>
       <c r="J23" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K23" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>66</v>
-      </c>
-      <c r="C24" t="s">
-        <v>67</v>
+        <v>46</v>
+      </c>
+      <c r="C24">
+        <v>213.42400000000001</v>
       </c>
       <c r="D24" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="E24" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F24">
         <v>3</v>
       </c>
       <c r="G24">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H24" t="s">
         <v>14</v>
@@ -1472,30 +1418,30 @@
         <v>16</v>
       </c>
       <c r="K24" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>68</v>
-      </c>
-      <c r="C25" t="s">
-        <v>69</v>
+        <v>47</v>
+      </c>
+      <c r="C25">
+        <v>220.34100000000001</v>
       </c>
       <c r="D25" t="s">
         <v>12</v>
       </c>
       <c r="E25" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F25">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G25">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H25" t="s">
         <v>14</v>
@@ -1504,48 +1450,16 @@
         <v>15</v>
       </c>
       <c r="J25" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="K25" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A26">
-        <v>25</v>
-      </c>
-      <c r="B26" t="s">
-        <v>70</v>
-      </c>
-      <c r="C26" t="s">
-        <v>71</v>
-      </c>
-      <c r="D26" t="s">
-        <v>12</v>
-      </c>
-      <c r="E26" t="s">
-        <v>20</v>
-      </c>
-      <c r="F26">
-        <v>0</v>
-      </c>
-      <c r="G26">
-        <v>0</v>
-      </c>
-      <c r="I26" t="s">
-        <v>15</v>
-      </c>
-      <c r="J26" t="s">
-        <v>17</v>
-      </c>
-      <c r="K26" t="s">
         <v>17</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:K3 A6:K6 A4:H4 J4:K4 A24:K26 A20:G20 J20:K20 A5:G5 J5:K5 A9:K9 A7:G7 J7:K7 A15:K16 A10:G10 J10:K10 A11:G11 J11:K11 A12:G12 J12:K12 A13:H13 J13:K13 A8:G8 I8:K8 A14:G14 I14:K14 A19:G19 A17:G17 I17:K17 A18:G18 I18:K18 I19:K19 A21:G21 I21:K21 A22:G22 I22:K22 A23:G23 I23:K23" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:K1 A6:C6 A2:C2 E2:K2 A3:C3 E3:K3 A4:C4 E4:K4 A5:C5 E5:K5 A25:K25 A24:C24 E24:J24 A17:K18 A13:J13 A9:K9 A7:C7 F7:K7 A23:C23 A22:C22 A21:K21 A19:C19 A20:J20 A14:C14 A15:C15 E6:K6 A8:C8 E8:K8 A11:K12 A10:C10 E10:K10 E14:J14 E15:J15 A16:C16 E16:K16 E19:J19 E23:J23 E22:J22" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>